<commit_message>
add-pdf-script-to read more information
</commit_message>
<xml_diff>
--- a/brushcustom询盘记录_updated.xlsx
+++ b/brushcustom询盘记录_updated.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R1e19830e65b44e62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rd726c617ba9f4900"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -433,6 +433,66 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">新加坡（提交地点）；公司位于瑞士 Zurich / Dietlikon</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Wasantha</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">imports@rhino.lk</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Upper Cleaning Brush Fibre 报价请求；数量 02 Nos；规格：fitted ø 350 / 254.75 x 1200 mm；要求 C&amp;F Colombo 报价，并提供品牌/原产国、技术数据表、图纸、交期、质保期和付款条款。附件 image002.jpg 为邮件签名/logo，非产品图纸。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Rhino Roofing Products Ltd.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">https://www.rhino.lk/</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">建筑材料/屋面和天花板材料制造（roofing &amp; ceiling sheets、金属屋面及配套产品）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">斯里兰卡 Colombo 09</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">有效询盘；需 C&amp;F Colombo 报价</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">D:\brushcustom-email-imap\attachments\2026-07-27_Rhino-Roofing-Products_Wasantha</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">David Burton</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">David.Burton@motion.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">RFQ 等效刷报价请求；客户询问能否按附件 PDF 图纸报价 equivalent brush。图纸信息：Brush, 60 inch, 0.04 inch NYLON；Part No. 5-050895；brush face width 54.00；hub-to-hub OD max / overall length 56.00；外径 ø10.00；内/芯部直径标注 ø1.94；原图纸来自 CP Manufacturing Inc.，Rev 1，日期 12/11/2006。默认公差/制造允许偏差（未特别说明时）：分数尺寸 ±0.06；一位小数 0.X ±0.1；两位小数 0.0X ±0.03；三位小数 0.00X ±0.01；整数角度 0° ±1°；一位小数角度 0.X° ±0.5°。图纸备注：shear and brake dimensions are O.D.；break all sharp edges, remove burrs。数量未给，需回信确认采购数量、材质/刷丝硬度、芯轴/端部结构、公差是否按原图执行和交付地址。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Motion</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">https://www.motion.com/</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">工业零部件/MRO 分销、机械动力传动、轴承、工业自动化及相关服务</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">大型企业（官网：600+ 北美网点、19 个分销中心）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">约 84 亿美元年销售额（2025，官网）</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">美国 California, Chula Vista；公司总部 Alabama, Birmingham</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">有效询盘；需按 PDF 图纸报等效刷，数量待确认</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">D:\brushcustom-email-imap\attachments\2026-07-30_Motion_David-Burton</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -504,7 +564,7 @@
       <x:name val="宋体"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -513,17 +573,22 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="7" tint="0.79989"/>
+        <x:fgColor theme="7" tint="0.79986"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="5" tint="0.79989"/>
+        <x:fgColor theme="5" tint="0.79986"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor theme="5" tint="0.79998"/>
+        <x:fgColor theme="5" tint="0.79995"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor theme="7" tint="0.79998"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -604,10 +669,10 @@
     <x:xf numFmtId="30" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="14" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="30" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -820,11 +885,11 @@
   <x:sheetFormatPr defaultRowHeight="16.5"/>
   <x:cols>
     <x:col min="1" max="1" width="12" style="5" customWidth="1"/>
-    <x:col min="2" max="2" width="17" style="5" customWidth="1"/>
-    <x:col min="3" max="3" width="28" style="5" customWidth="1"/>
+    <x:col min="2" max="2" width="10" style="5" customWidth="1"/>
+    <x:col min="3" max="3" width="22.75" style="5" customWidth="1"/>
     <x:col min="4" max="4" width="66" style="5" customWidth="1"/>
-    <x:col min="5" max="5" width="30" style="5" customWidth="1"/>
-    <x:col min="6" max="6" width="28" style="5" customWidth="1"/>
+    <x:col min="5" max="5" width="24.125" style="5" customWidth="1"/>
+    <x:col min="6" max="6" width="18.625" style="5" customWidth="1"/>
     <x:col min="7" max="7" width="36" style="5" customWidth="1"/>
     <x:col min="8" max="8" width="20" style="5" customWidth="1"/>
     <x:col min="9" max="9" width="20" style="10" customWidth="1"/>
@@ -1423,50 +1488,122 @@
       <x:c r="L16" s="11"/>
       <x:c r="M16" s="11"/>
     </x:row>
-    <x:row r="17" ht="118" customHeight="1">
-      <x:c r="A17" s="20" t="n">
+    <x:row r="17" ht="117.94999694824219" customHeight="1">
+      <x:c r="A17" s="19">
         <x:v>46230</x:v>
       </x:c>
-      <x:c r="B17" s="22" t="str">
-        <x:v>Wasantha</x:v>
-      </x:c>
-      <x:c r="C17" s="22" t="str">
-        <x:v>imports@rhino.lk</x:v>
-      </x:c>
-      <x:c r="D17" s="22" t="str">
-        <x:v>Upper Cleaning Brush Fibre 报价请求；数量 02 Nos；规格：fitted ø 350 / 254.75 x 1200 mm；要求 C&amp;F Colombo 报价，并提供品牌/原产国、技术数据表、图纸、交期、质保期和付款条款。附件 image002.jpg 为邮件签名/logo，非产品图纸。</x:v>
-      </x:c>
-      <x:c r="E17" s="22" t="str">
-        <x:v>Rhino Roofing Products Ltd.</x:v>
-      </x:c>
-      <x:c r="F17" s="22" t="str">
-        <x:v>https://www.rhino.lk/</x:v>
-      </x:c>
-      <x:c r="G17" s="22" t="str">
-        <x:v>建筑材料/屋面和天花板材料制造（roofing &amp; ceiling sheets、金属屋面及配套产品）</x:v>
-      </x:c>
-      <x:c r="H17" s="22" t="str">
+      <x:c r="B17" s="11" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="C17" s="11" t="s">
+        <x:v>140</x:v>
+      </x:c>
+      <x:c r="D17" s="11" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="E17" s="11" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="F17" s="11" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="G17" s="11" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="H17" s="11" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="I17" s="11" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="J17" s="11" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="K17" s="11" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="L17" s="11" t="s">
+        <x:v>147</x:v>
+      </x:c>
+      <x:c r="M17" s="11"/>
+    </x:row>
+    <x:row r="18" ht="150" customHeight="1">
+      <x:c r="A18" s="19">
+        <x:v>46233</x:v>
+      </x:c>
+      <x:c r="B18" s="11" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="C18" s="11" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="D18" s="11" t="s">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="E18" s="11" t="s">
+        <x:v>151</x:v>
+      </x:c>
+      <x:c r="F18" s="11" t="s">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="G18" s="11" t="s">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="H18" s="11" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="I18" s="11" t="s">
+        <x:v>155</x:v>
+      </x:c>
+      <x:c r="J18" s="11" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="K18" s="11" t="s">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="L18" s="11" t="s">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="M18" s="11"/>
+    </x:row>
+    <x:row r="19" ht="190" customHeight="1">
+      <x:c r="A19" s="20" t="n">
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="B19" s="22" t="str">
+        <x:v>Cherie Yeow</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="str">
+        <x:v>cherieyeow@neucorporation.com</x:v>
+      </x:c>
+      <x:c r="D19" s="22" t="str">
+        <x:v>Panel brush / BRUSH ASSEMBLY 报价请求；应用：半导体工厂设备/ESD 环境，安装在客户机器上。数量：评估 4 pcs，批准后每月至少 20 pcs/月。客户要求：PVC 底座；白色 ESD 刷丝，单根刷丝直径 0.07 mm。附件图纸信息：Title BRUSH ASSEMBLY；Part No./DWG No. N037-260608-A01；Rev A0；单位 MM；QTY 01 SET；Material TBA；主体尺寸约 168 x 42 x 30 mm；刷区/内框约 148 x 22 mm；Section B-B 显示底座/本体 15 mm、可见刷毛高度 15 mm、总高 30 mm、底部唇边 2 mm；横截面宽 42 mm；孔位/特征含 72x ø1 THRU、6x ø5 THRU、72x ø5 深/压装刷孔、4x R1.5，具体孔位按图纸。图纸备注：所有边倒角 0.10 [0.004]，未特别说明。一般公差：毫米 X ±0.5，X.X ±0.1，X.XX ±0.05，X.XXX ±0.020；英寸 .X ±.02，.XX ±.004，.XXX ±.002，.XXXX ±.0008；角度 X° ±1°，X.X° ±30'；粗糙度 Ra 0.8 µm。需报价 4pcs 和 20pcs，并确认 ESD 指标/PVC 等级/压装孔解释/交付地址。</x:v>
+      </x:c>
+      <x:c r="E19" s="22" t="str">
+        <x:v>NEU-PMC Pte Ltd</x:v>
+      </x:c>
+      <x:c r="F19" s="22" t="str">
         <x:v>待确认</x:v>
       </x:c>
-      <x:c r="I17" s="22" t="str">
+      <x:c r="G19" s="22" t="str">
+        <x:v>半导体装配/测试设备制造与维修；半导体工厂设备/ESD 应用</x:v>
+      </x:c>
+      <x:c r="H19" s="22" t="str">
+        <x:v>待确认（新加坡注册公司，2009 年成立；UEN 200907809Z）</x:v>
+      </x:c>
+      <x:c r="I19" s="22" t="str">
         <x:v>待确认</x:v>
       </x:c>
-      <x:c r="J17" s="22" t="str">
-        <x:v>斯里兰卡 Colombo 09</x:v>
-      </x:c>
-      <x:c r="K17" s="22" t="str">
-        <x:v>有效询盘；需 C&amp;F Colombo 报价</x:v>
-      </x:c>
-      <x:c r="L17" s="22" t="str">
-        <x:v>D:\brushcustom-email-imap\attachments\2026-07-27_Rhino-Roofing-Products_Wasantha</x:v>
-      </x:c>
-      <x:c r="M17" s="22" t="str"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="3"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="3"/>
+      <x:c r="J19" s="22" t="str">
+        <x:v>新加坡；公开注册地址为 2 Yishun Industrial Street 1 #03-29, North Point Bizhub, Singapore 768159</x:v>
+      </x:c>
+      <x:c r="K19" s="22" t="str">
+        <x:v>有效询盘；网站 RFQ 表单；有 PDF 图纸；需报价 4pcs 评估和 20pcs/月量产；官网/营收待确认</x:v>
+      </x:c>
+      <x:c r="L19" s="22" t="str">
+        <x:v>D:\brushcustom-email-imap\attachments\2026-08-01_NEU-PMC-Pte-Ltd_Cherie-Yeow</x:v>
+      </x:c>
+      <x:c r="M19" s="22" t="str"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="3"/>
@@ -1488,8 +1625,8 @@
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="R6c03b5aeb9e04bf3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="R4735b444ccb44883"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="R0c8f093a374544d9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="R5b6bc49154f34e3f"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>